<commit_message>
Update daily rainfall report
</commit_message>
<xml_diff>
--- a/rainfall_output/rainfall_2026-07-26.xlsx
+++ b/rainfall_output/rainfall_2026-07-26.xlsx
@@ -585,7 +585,9 @@
       <c r="D7" t="n">
         <v>74.64</v>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>34.1</v>
+      </c>
       <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -605,9 +607,7 @@
       <c r="D8" t="n">
         <v>74.89</v>
       </c>
-      <c r="E8" t="n">
-        <v>13.2</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>1.4</v>
       </c>
@@ -725,7 +725,9 @@
       <c r="D13" t="n">
         <v>74.09</v>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>32.6</v>
+      </c>
       <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -745,9 +747,7 @@
       <c r="D14" t="n">
         <v>73.58</v>
       </c>
-      <c r="E14" t="n">
-        <v>74.7</v>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
         <v>3.2</v>
       </c>
@@ -865,8 +865,12 @@
       <c r="D19" t="n">
         <v>75.77</v>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -885,12 +889,8 @@
       <c r="D20" t="n">
         <v>75.23999999999999</v>
       </c>
-      <c r="E20" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="F20" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1005,8 +1005,12 @@
       <c r="D25" t="n">
         <v>74.19</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3.9</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1028,9 +1032,7 @@
       <c r="E26" t="n">
         <v>13.4</v>
       </c>
-      <c r="F26" t="n">
-        <v>0.8</v>
-      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1052,9 +1054,7 @@
       <c r="E27" t="n">
         <v>23.2</v>
       </c>
-      <c r="F27" t="n">
-        <v>2.7</v>
-      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1073,9 +1073,7 @@
       <c r="D28" t="n">
         <v>74.08</v>
       </c>
-      <c r="E28" t="n">
-        <v>34.2</v>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
         <v>0.5</v>
       </c>
@@ -1145,8 +1143,12 @@
       <c r="D31" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1192,9 +1194,7 @@
       <c r="E33" t="n">
         <v>36.1</v>
       </c>
-      <c r="F33" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1216,9 +1216,7 @@
       <c r="E34" t="n">
         <v>24.4</v>
       </c>
-      <c r="F34" t="n">
-        <v>2.2</v>
-      </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1237,9 +1235,7 @@
       <c r="D35" t="n">
         <v>74.36</v>
       </c>
-      <c r="E35" t="n">
-        <v>31.6</v>
-      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
         <v>3.6</v>
       </c>
@@ -1288,7 +1284,9 @@
       <c r="E37" t="n">
         <v>32.5</v>
       </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1307,7 +1305,9 @@
       <c r="D38" t="n">
         <v>77.11</v>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>10.7</v>
+      </c>
       <c r="F38" t="n">
         <v>0.7</v>
       </c>
@@ -1356,9 +1356,7 @@
       <c r="E40" t="n">
         <v>6.6</v>
       </c>
-      <c r="F40" t="n">
-        <v>17.3</v>
-      </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1377,9 +1375,7 @@
       <c r="D41" t="n">
         <v>75.91</v>
       </c>
-      <c r="E41" t="n">
-        <v>17.6</v>
-      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
         <v>1.6</v>
       </c>
@@ -1449,8 +1445,12 @@
       <c r="D44" t="n">
         <v>75.14</v>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4.9</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">

</xml_diff>